<commit_message>
backup att dia 11
</commit_message>
<xml_diff>
--- a/perfil/templates/planilhas/ficha_colab.xlsx
+++ b/perfil/templates/planilhas/ficha_colab.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pichau\Desktop\PROJETOS\SISTEMA_CONTROLE_COMERCIAL\perfil\templates\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B8577A-CCD5-4D3A-ADFE-AE5A78666C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB14CC40-ACC9-46A9-9277-574CAD52D122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9075" yWindow="7260" windowWidth="18750" windowHeight="8220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="128">
   <si>
     <t>FICHA DE FUNCIONÁRIO -  ADMISSÃO</t>
   </si>
@@ -190,9 +190,6 @@
     <t>R.G.:</t>
   </si>
   <si>
-    <t xml:space="preserve">UF: </t>
-  </si>
-  <si>
     <t>Orgão Expedidor:</t>
   </si>
   <si>
@@ -425,6 +422,12 @@
   </si>
   <si>
     <t>ok</t>
+  </si>
+  <si>
+    <t>REMOVER</t>
+  </si>
+  <si>
+    <t>remover</t>
   </si>
 </sst>
 </file>
@@ -1420,342 +1423,46 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="2" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1764,48 +1471,344 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="2" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2092,7 +2095,8 @@
   <cols>
     <col min="1" max="1" width="7.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="7.140625" style="1" customWidth="1"/>
-    <col min="3" max="7" width="8" style="1" customWidth="1"/>
+    <col min="3" max="6" width="8" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="1" customWidth="1"/>
     <col min="9" max="16" width="8" style="1" customWidth="1"/>
     <col min="17" max="256" width="9.140625" style="1"/>
@@ -2477,13 +2481,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="234"/>
-      <c r="C1" s="234"/>
-      <c r="D1" s="234"/>
-      <c r="E1" s="234"/>
-      <c r="F1" s="234"/>
-      <c r="G1" s="234"/>
-      <c r="H1" s="234"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
@@ -2493,16 +2497,16 @@
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="234" t="s">
+      <c r="B2" s="108" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="234"/>
-      <c r="D2" s="234"/>
-      <c r="E2" s="234"/>
-      <c r="F2" s="234"/>
-      <c r="G2" s="234"/>
-      <c r="H2" s="234"/>
-      <c r="I2" s="234"/>
+      <c r="C2" s="108"/>
+      <c r="D2" s="108"/>
+      <c r="E2" s="108"/>
+      <c r="F2" s="108"/>
+      <c r="G2" s="108"/>
+      <c r="H2" s="108"/>
+      <c r="I2" s="108"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -2524,26 +2528,26 @@
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:16" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="235" t="s">
+      <c r="A5" s="109" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="236"/>
-      <c r="C5" s="118" t="s">
-        <v>125</v>
-      </c>
-      <c r="D5" s="119"/>
-      <c r="E5" s="119"/>
-      <c r="F5" s="119"/>
-      <c r="G5" s="119"/>
-      <c r="H5" s="119"/>
-      <c r="I5" s="119"/>
-      <c r="J5" s="119"/>
-      <c r="K5" s="119"/>
-      <c r="L5" s="119"/>
-      <c r="M5" s="119"/>
-      <c r="N5" s="119"/>
-      <c r="O5" s="119"/>
-      <c r="P5" s="120"/>
+      <c r="B5" s="110"/>
+      <c r="C5" s="231" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="232"/>
+      <c r="E5" s="232"/>
+      <c r="F5" s="232"/>
+      <c r="G5" s="232"/>
+      <c r="H5" s="232"/>
+      <c r="I5" s="232"/>
+      <c r="J5" s="232"/>
+      <c r="K5" s="232"/>
+      <c r="L5" s="232"/>
+      <c r="M5" s="232"/>
+      <c r="N5" s="232"/>
+      <c r="O5" s="232"/>
+      <c r="P5" s="233"/>
     </row>
     <row r="6" spans="1:16" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="3"/>
@@ -2562,149 +2566,149 @@
       <c r="P6" s="3"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="135" t="s">
+      <c r="A7" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="136"/>
-      <c r="C7" s="136"/>
-      <c r="D7" s="136"/>
-      <c r="E7" s="136"/>
-      <c r="F7" s="136"/>
-      <c r="G7" s="136"/>
-      <c r="H7" s="136"/>
-      <c r="I7" s="136"/>
-      <c r="J7" s="136"/>
-      <c r="K7" s="136"/>
-      <c r="L7" s="136"/>
-      <c r="M7" s="136"/>
-      <c r="N7" s="136"/>
-      <c r="O7" s="136"/>
-      <c r="P7" s="137"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="112"/>
+      <c r="D7" s="112"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="112"/>
+      <c r="G7" s="112"/>
+      <c r="H7" s="112"/>
+      <c r="I7" s="112"/>
+      <c r="J7" s="112"/>
+      <c r="K7" s="112"/>
+      <c r="L7" s="112"/>
+      <c r="M7" s="112"/>
+      <c r="N7" s="112"/>
+      <c r="O7" s="112"/>
+      <c r="P7" s="113"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="162" t="s">
+      <c r="A8" s="114" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="199"/>
-      <c r="C8" s="237" t="s">
-        <v>126</v>
-      </c>
-      <c r="D8" s="238"/>
-      <c r="E8" s="238"/>
-      <c r="F8" s="238"/>
-      <c r="G8" s="238"/>
-      <c r="H8" s="238"/>
-      <c r="I8" s="238"/>
-      <c r="J8" s="238"/>
-      <c r="K8" s="238"/>
-      <c r="L8" s="238"/>
-      <c r="M8" s="238"/>
-      <c r="N8" s="238"/>
-      <c r="O8" s="238"/>
-      <c r="P8" s="239"/>
+      <c r="B8" s="115"/>
+      <c r="C8" s="116" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="117"/>
+      <c r="E8" s="117"/>
+      <c r="F8" s="117"/>
+      <c r="G8" s="117"/>
+      <c r="H8" s="117"/>
+      <c r="I8" s="117"/>
+      <c r="J8" s="117"/>
+      <c r="K8" s="117"/>
+      <c r="L8" s="117"/>
+      <c r="M8" s="117"/>
+      <c r="N8" s="117"/>
+      <c r="O8" s="117"/>
+      <c r="P8" s="118"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="138" t="s">
+      <c r="A9" s="137" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="213"/>
-      <c r="C9" s="230" t="s">
-        <v>126</v>
-      </c>
-      <c r="D9" s="230"/>
-      <c r="E9" s="230"/>
-      <c r="F9" s="230"/>
-      <c r="G9" s="230"/>
-      <c r="H9" s="230"/>
-      <c r="I9" s="230"/>
-      <c r="J9" s="230"/>
-      <c r="K9" s="230"/>
-      <c r="L9" s="230"/>
-      <c r="M9" s="230"/>
-      <c r="N9" s="230"/>
+      <c r="B9" s="138"/>
+      <c r="C9" s="139" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="139"/>
+      <c r="E9" s="139"/>
+      <c r="F9" s="139"/>
+      <c r="G9" s="139"/>
+      <c r="H9" s="139"/>
+      <c r="I9" s="139"/>
+      <c r="J9" s="139"/>
+      <c r="K9" s="139"/>
+      <c r="L9" s="139"/>
+      <c r="M9" s="139"/>
+      <c r="N9" s="139"/>
       <c r="O9" s="6" t="s">
         <v>6</v>
       </c>
       <c r="P9" s="7"/>
     </row>
     <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="108" t="s">
+      <c r="A10" s="121" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="222"/>
-      <c r="C10" s="231"/>
-      <c r="D10" s="142"/>
-      <c r="E10" s="174"/>
+      <c r="B10" s="122"/>
+      <c r="C10" s="140"/>
+      <c r="D10" s="141"/>
+      <c r="E10" s="142"/>
       <c r="F10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="142" t="s">
-        <v>126</v>
-      </c>
-      <c r="H10" s="142"/>
-      <c r="I10" s="142"/>
-      <c r="J10" s="142"/>
-      <c r="K10" s="142"/>
-      <c r="L10" s="174"/>
+      <c r="G10" s="141" t="s">
+        <v>125</v>
+      </c>
+      <c r="H10" s="141"/>
+      <c r="I10" s="141"/>
+      <c r="J10" s="141"/>
+      <c r="K10" s="141"/>
+      <c r="L10" s="142"/>
       <c r="M10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="N10" s="232" t="s">
-        <v>126</v>
-      </c>
-      <c r="O10" s="232"/>
-      <c r="P10" s="233"/>
+      <c r="N10" s="143" t="s">
+        <v>125</v>
+      </c>
+      <c r="O10" s="143"/>
+      <c r="P10" s="144"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="108" t="s">
+      <c r="A11" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="222"/>
-      <c r="C11" s="223" t="s">
-        <v>126</v>
-      </c>
-      <c r="D11" s="224"/>
-      <c r="E11" s="224"/>
-      <c r="F11" s="224"/>
-      <c r="G11" s="224"/>
-      <c r="H11" s="225"/>
+      <c r="B11" s="122"/>
+      <c r="C11" s="123" t="s">
+        <v>125</v>
+      </c>
+      <c r="D11" s="124"/>
+      <c r="E11" s="124"/>
+      <c r="F11" s="124"/>
+      <c r="G11" s="124"/>
+      <c r="H11" s="125"/>
       <c r="I11" s="126" t="s">
         <v>11</v>
       </c>
-      <c r="J11" s="109"/>
-      <c r="K11" s="224" t="s">
-        <v>126</v>
-      </c>
-      <c r="L11" s="224"/>
-      <c r="M11" s="224"/>
-      <c r="N11" s="224"/>
-      <c r="O11" s="224"/>
-      <c r="P11" s="226"/>
+      <c r="J11" s="127"/>
+      <c r="K11" s="124" t="s">
+        <v>125</v>
+      </c>
+      <c r="L11" s="124"/>
+      <c r="M11" s="124"/>
+      <c r="N11" s="124"/>
+      <c r="O11" s="124"/>
+      <c r="P11" s="128"/>
     </row>
     <row r="12" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="216" t="s">
+      <c r="A12" s="129" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="217"/>
-      <c r="C12" s="227" t="s">
-        <v>126</v>
-      </c>
-      <c r="D12" s="212"/>
-      <c r="E12" s="218"/>
-      <c r="F12" s="228" t="s">
+      <c r="B12" s="130"/>
+      <c r="C12" s="131" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="132"/>
+      <c r="E12" s="133"/>
+      <c r="F12" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="229"/>
-      <c r="H12" s="205" t="s">
-        <v>126</v>
-      </c>
-      <c r="I12" s="205"/>
-      <c r="J12" s="205"/>
+      <c r="G12" s="135"/>
+      <c r="H12" s="136" t="s">
+        <v>125</v>
+      </c>
+      <c r="I12" s="136"/>
+      <c r="J12" s="136"/>
       <c r="K12" s="15" t="s">
         <v>14</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M12" s="14" t="s">
         <v>15</v>
@@ -2714,134 +2718,134 @@
       <c r="P12" s="17"/>
     </row>
     <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="138" t="s">
+      <c r="A13" s="137" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="213"/>
-      <c r="C13" s="201" t="s">
-        <v>126</v>
-      </c>
-      <c r="D13" s="214"/>
-      <c r="E13" s="214"/>
-      <c r="F13" s="214"/>
-      <c r="G13" s="214"/>
-      <c r="H13" s="214"/>
-      <c r="I13" s="214"/>
-      <c r="J13" s="214"/>
-      <c r="K13" s="214"/>
-      <c r="L13" s="214"/>
-      <c r="M13" s="214"/>
-      <c r="N13" s="214"/>
-      <c r="O13" s="214"/>
-      <c r="P13" s="215"/>
+      <c r="B13" s="138"/>
+      <c r="C13" s="152" t="s">
+        <v>125</v>
+      </c>
+      <c r="D13" s="153"/>
+      <c r="E13" s="153"/>
+      <c r="F13" s="153"/>
+      <c r="G13" s="153"/>
+      <c r="H13" s="153"/>
+      <c r="I13" s="153"/>
+      <c r="J13" s="153"/>
+      <c r="K13" s="153"/>
+      <c r="L13" s="153"/>
+      <c r="M13" s="153"/>
+      <c r="N13" s="153"/>
+      <c r="O13" s="153"/>
+      <c r="P13" s="154"/>
     </row>
     <row r="14" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="216" t="s">
+      <c r="A14" s="129" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="217"/>
-      <c r="C14" s="218" t="s">
-        <v>126</v>
-      </c>
-      <c r="D14" s="219"/>
-      <c r="E14" s="219"/>
-      <c r="F14" s="219"/>
-      <c r="G14" s="219"/>
-      <c r="H14" s="219"/>
-      <c r="I14" s="219"/>
-      <c r="J14" s="219"/>
-      <c r="K14" s="219"/>
-      <c r="L14" s="219"/>
-      <c r="M14" s="219"/>
-      <c r="N14" s="219"/>
-      <c r="O14" s="219"/>
-      <c r="P14" s="220"/>
+      <c r="B14" s="130"/>
+      <c r="C14" s="133" t="s">
+        <v>125</v>
+      </c>
+      <c r="D14" s="155"/>
+      <c r="E14" s="155"/>
+      <c r="F14" s="155"/>
+      <c r="G14" s="155"/>
+      <c r="H14" s="155"/>
+      <c r="I14" s="155"/>
+      <c r="J14" s="155"/>
+      <c r="K14" s="155"/>
+      <c r="L14" s="155"/>
+      <c r="M14" s="155"/>
+      <c r="N14" s="155"/>
+      <c r="O14" s="155"/>
+      <c r="P14" s="156"/>
     </row>
     <row r="15" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="221" t="s">
+      <c r="A15" s="157" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="211"/>
-      <c r="C15" s="121"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="B15" s="151"/>
+      <c r="C15" s="234"/>
+      <c r="D15" s="203"/>
+      <c r="E15" s="235"/>
       <c r="F15" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="121"/>
-      <c r="H15" s="122"/>
-      <c r="I15" s="123"/>
+      <c r="G15" s="234"/>
+      <c r="H15" s="203"/>
+      <c r="I15" s="235"/>
       <c r="J15" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="K15" s="122"/>
-      <c r="L15" s="122"/>
-      <c r="M15" s="123"/>
+      <c r="K15" s="203"/>
+      <c r="L15" s="203"/>
+      <c r="M15" s="235"/>
       <c r="N15" s="20"/>
       <c r="O15" s="20"/>
       <c r="P15" s="21"/>
     </row>
     <row r="16" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="191" t="s">
+      <c r="A16" s="145" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="206"/>
+      <c r="B16" s="146"/>
       <c r="C16" s="22" t="s">
-        <v>126</v>
-      </c>
-      <c r="D16" s="209" t="s">
+        <v>125</v>
+      </c>
+      <c r="D16" s="149" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="209"/>
-      <c r="F16" s="209"/>
+      <c r="E16" s="149"/>
+      <c r="F16" s="149"/>
       <c r="G16" s="24"/>
-      <c r="H16" s="209" t="s">
+      <c r="H16" s="149" t="s">
         <v>23</v>
       </c>
-      <c r="I16" s="209"/>
+      <c r="I16" s="149"/>
       <c r="J16" s="25"/>
-      <c r="K16" s="210" t="s">
+      <c r="K16" s="150" t="s">
         <v>24</v>
       </c>
-      <c r="L16" s="210"/>
+      <c r="L16" s="150"/>
       <c r="M16" s="26"/>
-      <c r="N16" s="210" t="s">
+      <c r="N16" s="150" t="s">
         <v>25</v>
       </c>
-      <c r="O16" s="210"/>
-      <c r="P16" s="211"/>
+      <c r="O16" s="150"/>
+      <c r="P16" s="151"/>
     </row>
     <row r="17" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="207"/>
-      <c r="B17" s="208"/>
+      <c r="A17" s="147"/>
+      <c r="B17" s="148"/>
       <c r="C17" s="27"/>
-      <c r="D17" s="209" t="s">
+      <c r="D17" s="149" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="209"/>
+      <c r="E17" s="149"/>
       <c r="F17" s="28"/>
-      <c r="G17" s="209" t="s">
+      <c r="G17" s="149" t="s">
         <v>27</v>
       </c>
-      <c r="H17" s="209"/>
+      <c r="H17" s="149"/>
       <c r="I17" s="24"/>
       <c r="J17" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="K17" s="184"/>
-      <c r="L17" s="184"/>
-      <c r="M17" s="184"/>
-      <c r="N17" s="184"/>
-      <c r="O17" s="184"/>
-      <c r="P17" s="240"/>
+      <c r="K17" s="119"/>
+      <c r="L17" s="119"/>
+      <c r="M17" s="119"/>
+      <c r="N17" s="119"/>
+      <c r="O17" s="119"/>
+      <c r="P17" s="120"/>
     </row>
     <row r="18" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="162" t="s">
+      <c r="A18" s="114" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="199"/>
+      <c r="B18" s="115"/>
       <c r="C18" s="29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D18" s="30" t="s">
         <v>30</v>
@@ -2855,60 +2859,70 @@
         <v>32</v>
       </c>
       <c r="I18" s="24"/>
-      <c r="J18" s="190" t="s">
+      <c r="J18" s="158" t="s">
         <v>33</v>
       </c>
-      <c r="K18" s="190"/>
-      <c r="L18" s="190"/>
+      <c r="K18" s="158"/>
+      <c r="L18" s="158"/>
       <c r="M18" s="24"/>
-      <c r="N18" s="190" t="s">
+      <c r="N18" s="158" t="s">
         <v>34</v>
       </c>
-      <c r="O18" s="190"/>
-      <c r="P18" s="200"/>
+      <c r="O18" s="158"/>
+      <c r="P18" s="159"/>
     </row>
     <row r="19" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="193" t="s">
+      <c r="A19" s="160" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="194"/>
+      <c r="B19" s="161"/>
       <c r="C19" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="177"/>
-      <c r="E19" s="177"/>
-      <c r="F19" s="177"/>
-      <c r="G19" s="177"/>
-      <c r="H19" s="177"/>
-      <c r="I19" s="177"/>
-      <c r="J19" s="177"/>
-      <c r="K19" s="177"/>
-      <c r="L19" s="201"/>
-      <c r="M19" s="156" t="s">
+      <c r="D19" s="164" t="s">
+        <v>125</v>
+      </c>
+      <c r="E19" s="164"/>
+      <c r="F19" s="164"/>
+      <c r="G19" s="164"/>
+      <c r="H19" s="164"/>
+      <c r="I19" s="164"/>
+      <c r="J19" s="164"/>
+      <c r="K19" s="164"/>
+      <c r="L19" s="152"/>
+      <c r="M19" s="165" t="s">
         <v>36</v>
       </c>
-      <c r="N19" s="157"/>
-      <c r="O19" s="198"/>
-      <c r="P19" s="202"/>
+      <c r="N19" s="166"/>
+      <c r="O19" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="P19" s="168"/>
     </row>
     <row r="20" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="195"/>
-      <c r="B20" s="196"/>
+      <c r="A20" s="162"/>
+      <c r="B20" s="163"/>
       <c r="C20" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="203"/>
-      <c r="E20" s="204"/>
+      <c r="D20" s="169" t="s">
+        <v>125</v>
+      </c>
+      <c r="E20" s="170"/>
       <c r="F20" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="G20" s="36"/>
+      <c r="G20" s="36" t="s">
+        <v>126</v>
+      </c>
       <c r="H20" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="I20" s="205"/>
-      <c r="J20" s="205"/>
-      <c r="K20" s="205"/>
+      <c r="I20" s="136" t="s">
+        <v>125</v>
+      </c>
+      <c r="J20" s="136"/>
+      <c r="K20" s="136"/>
       <c r="L20" s="37"/>
       <c r="M20" s="38"/>
       <c r="N20" s="38"/>
@@ -2916,100 +2930,100 @@
       <c r="P20" s="39"/>
     </row>
     <row r="21" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="191" t="s">
+      <c r="A21" s="145" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="192"/>
+      <c r="B21" s="177"/>
       <c r="C21" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="197"/>
-      <c r="E21" s="197"/>
-      <c r="F21" s="197"/>
-      <c r="G21" s="197"/>
-      <c r="H21" s="141"/>
-      <c r="I21" s="156" t="s">
+      <c r="D21" s="178"/>
+      <c r="E21" s="178"/>
+      <c r="F21" s="178"/>
+      <c r="G21" s="178"/>
+      <c r="H21" s="179"/>
+      <c r="I21" s="165" t="s">
         <v>36</v>
       </c>
-      <c r="J21" s="157"/>
-      <c r="K21" s="198"/>
-      <c r="L21" s="198"/>
-      <c r="M21" s="176" t="s">
+      <c r="J21" s="166"/>
+      <c r="K21" s="167"/>
+      <c r="L21" s="167"/>
+      <c r="M21" s="180" t="s">
         <v>42</v>
       </c>
-      <c r="N21" s="139"/>
+      <c r="N21" s="181"/>
       <c r="O21" s="41"/>
       <c r="P21" s="42"/>
     </row>
     <row r="22" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="193"/>
-      <c r="B22" s="194"/>
+      <c r="A22" s="160"/>
+      <c r="B22" s="161"/>
       <c r="C22" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D22" s="124"/>
-      <c r="E22" s="124"/>
-      <c r="F22" s="124"/>
-      <c r="G22" s="124"/>
-      <c r="H22" s="125"/>
+      <c r="D22" s="182"/>
+      <c r="E22" s="182"/>
+      <c r="F22" s="182"/>
+      <c r="G22" s="182"/>
+      <c r="H22" s="183"/>
       <c r="I22" s="126" t="s">
         <v>36</v>
       </c>
-      <c r="J22" s="109"/>
-      <c r="K22" s="183"/>
-      <c r="L22" s="183"/>
-      <c r="M22" s="156" t="s">
+      <c r="J22" s="127"/>
+      <c r="K22" s="171"/>
+      <c r="L22" s="171"/>
+      <c r="M22" s="165" t="s">
         <v>42</v>
       </c>
-      <c r="N22" s="157"/>
+      <c r="N22" s="166"/>
       <c r="O22" s="43"/>
       <c r="P22" s="44"/>
     </row>
     <row r="23" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="193"/>
-      <c r="B23" s="194"/>
+      <c r="A23" s="160"/>
+      <c r="B23" s="161"/>
       <c r="C23" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="124"/>
-      <c r="E23" s="124"/>
-      <c r="F23" s="124"/>
-      <c r="G23" s="124"/>
-      <c r="H23" s="125"/>
-      <c r="I23" s="156" t="s">
+      <c r="D23" s="182"/>
+      <c r="E23" s="182"/>
+      <c r="F23" s="182"/>
+      <c r="G23" s="182"/>
+      <c r="H23" s="183"/>
+      <c r="I23" s="165" t="s">
         <v>36</v>
       </c>
-      <c r="J23" s="157"/>
-      <c r="K23" s="183"/>
-      <c r="L23" s="183"/>
-      <c r="M23" s="156" t="s">
+      <c r="J23" s="166"/>
+      <c r="K23" s="171"/>
+      <c r="L23" s="171"/>
+      <c r="M23" s="165" t="s">
         <v>42</v>
       </c>
-      <c r="N23" s="157"/>
+      <c r="N23" s="166"/>
       <c r="O23" s="43"/>
       <c r="P23" s="44"/>
     </row>
     <row r="24" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="195"/>
-      <c r="B24" s="196"/>
+      <c r="A24" s="162"/>
+      <c r="B24" s="163"/>
       <c r="C24" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="184"/>
-      <c r="E24" s="184"/>
-      <c r="F24" s="184"/>
-      <c r="G24" s="184"/>
-      <c r="H24" s="185"/>
-      <c r="I24" s="186" t="s">
+      <c r="D24" s="119"/>
+      <c r="E24" s="119"/>
+      <c r="F24" s="119"/>
+      <c r="G24" s="119"/>
+      <c r="H24" s="172"/>
+      <c r="I24" s="173" t="s">
         <v>36</v>
       </c>
-      <c r="J24" s="187"/>
-      <c r="K24" s="188"/>
-      <c r="L24" s="188"/>
-      <c r="M24" s="189" t="s">
+      <c r="J24" s="174"/>
+      <c r="K24" s="175"/>
+      <c r="L24" s="175"/>
+      <c r="M24" s="176" t="s">
         <v>42</v>
       </c>
-      <c r="N24" s="190"/>
+      <c r="N24" s="158"/>
       <c r="O24" s="46"/>
       <c r="P24" s="47"/>
     </row>
@@ -3031,181 +3045,216 @@
       <c r="P25" s="49"/>
     </row>
     <row r="26" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="135" t="s">
+      <c r="A26" s="111" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="136"/>
-      <c r="C26" s="136"/>
-      <c r="D26" s="136"/>
-      <c r="E26" s="136"/>
-      <c r="F26" s="136"/>
-      <c r="G26" s="136"/>
-      <c r="H26" s="136"/>
-      <c r="I26" s="136"/>
-      <c r="J26" s="136"/>
-      <c r="K26" s="136"/>
-      <c r="L26" s="136"/>
-      <c r="M26" s="136"/>
-      <c r="N26" s="136"/>
-      <c r="O26" s="136"/>
-      <c r="P26" s="137"/>
+      <c r="B26" s="112"/>
+      <c r="C26" s="112"/>
+      <c r="D26" s="112"/>
+      <c r="E26" s="112"/>
+      <c r="F26" s="112"/>
+      <c r="G26" s="112"/>
+      <c r="H26" s="112"/>
+      <c r="I26" s="112"/>
+      <c r="J26" s="112"/>
+      <c r="K26" s="112"/>
+      <c r="L26" s="112"/>
+      <c r="M26" s="112"/>
+      <c r="N26" s="112"/>
+      <c r="O26" s="112"/>
+      <c r="P26" s="113"/>
     </row>
     <row r="27" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="175"/>
-      <c r="C27" s="175"/>
-      <c r="D27" s="176" t="s">
+      <c r="B27" s="188" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="188"/>
+      <c r="D27" s="180" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="139"/>
-      <c r="F27" s="177"/>
-      <c r="G27" s="177"/>
+      <c r="E27" s="181"/>
+      <c r="F27" s="164" t="s">
+        <v>125</v>
+      </c>
+      <c r="G27" s="164"/>
       <c r="H27" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="J27" s="178" t="s">
+      <c r="I27" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="J27" s="189" t="s">
         <v>46</v>
       </c>
-      <c r="K27" s="179"/>
-      <c r="L27" s="140"/>
-      <c r="M27" s="180"/>
+      <c r="K27" s="190"/>
+      <c r="L27" s="191" t="s">
+        <v>125</v>
+      </c>
+      <c r="M27" s="192"/>
       <c r="N27" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="O27" s="181"/>
-      <c r="P27" s="182"/>
+      <c r="O27" s="193"/>
+      <c r="P27" s="194"/>
     </row>
     <row r="28" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B28" s="172"/>
-      <c r="C28" s="124"/>
-      <c r="D28" s="124"/>
+      <c r="B28" s="184" t="s">
+        <v>125</v>
+      </c>
+      <c r="C28" s="182"/>
+      <c r="D28" s="182"/>
       <c r="E28" s="10" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="F28" s="43"/>
       <c r="G28" s="126" t="s">
+        <v>49</v>
+      </c>
+      <c r="H28" s="127"/>
+      <c r="I28" s="182" t="s">
+        <v>125</v>
+      </c>
+      <c r="J28" s="183"/>
+      <c r="K28" s="126" t="s">
         <v>50</v>
       </c>
-      <c r="H28" s="109"/>
-      <c r="I28" s="124"/>
-      <c r="J28" s="125"/>
-      <c r="K28" s="126" t="s">
-        <v>51</v>
-      </c>
-      <c r="L28" s="157"/>
-      <c r="M28" s="157"/>
-      <c r="N28" s="170"/>
-      <c r="O28" s="170"/>
-      <c r="P28" s="171"/>
+      <c r="L28" s="166"/>
+      <c r="M28" s="166"/>
+      <c r="N28" s="185" t="s">
+        <v>125</v>
+      </c>
+      <c r="O28" s="185"/>
+      <c r="P28" s="186"/>
     </row>
     <row r="29" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="173"/>
-      <c r="C29" s="173"/>
-      <c r="D29" s="173"/>
-      <c r="E29" s="173"/>
-      <c r="F29" s="109" t="s">
+      <c r="B29" s="187" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" s="187"/>
+      <c r="D29" s="187"/>
+      <c r="E29" s="187"/>
+      <c r="F29" s="127" t="s">
+        <v>51</v>
+      </c>
+      <c r="G29" s="127"/>
+      <c r="H29" s="141" t="s">
+        <v>125</v>
+      </c>
+      <c r="I29" s="141"/>
+      <c r="J29" s="141"/>
+      <c r="K29" s="141"/>
+      <c r="L29" s="141"/>
+      <c r="M29" s="141"/>
+      <c r="N29" s="141"/>
+      <c r="O29" s="141"/>
+      <c r="P29" s="142"/>
+    </row>
+    <row r="30" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="195" t="s">
         <v>52</v>
       </c>
-      <c r="G29" s="109"/>
-      <c r="H29" s="142"/>
-      <c r="I29" s="142"/>
-      <c r="J29" s="142"/>
-      <c r="K29" s="142"/>
-      <c r="L29" s="142"/>
-      <c r="M29" s="142"/>
-      <c r="N29" s="142"/>
-      <c r="O29" s="142"/>
-      <c r="P29" s="174"/>
-    </row>
-    <row r="30" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="168" t="s">
+      <c r="B30" s="166"/>
+      <c r="C30" s="196" t="s">
+        <v>125</v>
+      </c>
+      <c r="D30" s="196"/>
+      <c r="E30" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="157"/>
-      <c r="C30" s="169"/>
-      <c r="D30" s="169"/>
-      <c r="E30" s="53" t="s">
+      <c r="F30" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="G30" s="9" t="s">
         <v>54</v>
-      </c>
-      <c r="F30" s="12"/>
-      <c r="G30" s="9" t="s">
-        <v>55</v>
       </c>
       <c r="H30" s="8"/>
       <c r="I30" s="126" t="s">
-        <v>56</v>
-      </c>
-      <c r="J30" s="109"/>
-      <c r="K30" s="142"/>
-      <c r="L30" s="142"/>
+        <v>55</v>
+      </c>
+      <c r="J30" s="127"/>
+      <c r="K30" s="141"/>
+      <c r="L30" s="141"/>
       <c r="M30" s="11"/>
       <c r="N30" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="O30" s="170"/>
-      <c r="P30" s="171"/>
+        <v>56</v>
+      </c>
+      <c r="O30" s="185" t="s">
+        <v>127</v>
+      </c>
+      <c r="P30" s="186"/>
     </row>
     <row r="31" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="127" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="109" t="s">
+      <c r="C31" s="127"/>
+      <c r="D31" s="182"/>
+      <c r="E31" s="183"/>
+      <c r="F31" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="109"/>
-      <c r="D31" s="124"/>
-      <c r="E31" s="125"/>
-      <c r="F31" s="10" t="s">
+      <c r="G31" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="H31" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="54" t="s">
+      <c r="I31" s="185" t="s">
+        <v>125</v>
+      </c>
+      <c r="J31" s="186"/>
+      <c r="K31" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I31" s="170"/>
-      <c r="J31" s="171"/>
-      <c r="K31" s="10" t="s">
+      <c r="L31" s="185" t="s">
+        <v>127</v>
+      </c>
+      <c r="M31" s="185"/>
+      <c r="N31" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="O31" s="185" t="s">
+        <v>127</v>
+      </c>
+      <c r="P31" s="186"/>
+    </row>
+    <row r="32" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="165" t="s">
         <v>62</v>
       </c>
-      <c r="L31" s="170"/>
-      <c r="M31" s="170"/>
-      <c r="N31" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="O31" s="170"/>
-      <c r="P31" s="171"/>
-    </row>
-    <row r="32" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="156" t="s">
-        <v>63</v>
-      </c>
-      <c r="B32" s="109"/>
-      <c r="C32" s="160"/>
-      <c r="D32" s="124"/>
-      <c r="E32" s="125"/>
-      <c r="F32" s="161"/>
-      <c r="G32" s="142"/>
-      <c r="H32" s="124"/>
-      <c r="I32" s="124"/>
-      <c r="J32" s="124"/>
-      <c r="K32" s="124"/>
-      <c r="L32" s="124"/>
-      <c r="M32" s="124"/>
-      <c r="N32" s="124"/>
-      <c r="O32" s="124"/>
-      <c r="P32" s="125"/>
+      <c r="B32" s="127"/>
+      <c r="C32" s="197" t="s">
+        <v>125</v>
+      </c>
+      <c r="D32" s="182"/>
+      <c r="E32" s="183"/>
+      <c r="F32" s="198"/>
+      <c r="G32" s="141"/>
+      <c r="H32" s="182"/>
+      <c r="I32" s="182"/>
+      <c r="J32" s="182"/>
+      <c r="K32" s="182"/>
+      <c r="L32" s="182"/>
+      <c r="M32" s="182"/>
+      <c r="N32" s="182"/>
+      <c r="O32" s="182"/>
+      <c r="P32" s="183"/>
     </row>
     <row r="33" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="52" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B33" s="50"/>
       <c r="C33" s="55"/>
@@ -3224,54 +3273,64 @@
       <c r="P33" s="34"/>
     </row>
     <row r="34" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="135" t="s">
+      <c r="A34" s="111" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="112"/>
+      <c r="C34" s="112"/>
+      <c r="D34" s="112"/>
+      <c r="E34" s="112"/>
+      <c r="F34" s="112"/>
+      <c r="G34" s="112"/>
+      <c r="H34" s="112"/>
+      <c r="I34" s="199"/>
+      <c r="J34" s="199"/>
+      <c r="K34" s="112"/>
+      <c r="L34" s="112"/>
+      <c r="M34" s="112"/>
+      <c r="N34" s="112"/>
+      <c r="O34" s="112"/>
+      <c r="P34" s="113"/>
+    </row>
+    <row r="35" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="114" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="136"/>
-      <c r="C34" s="136"/>
-      <c r="D34" s="136"/>
-      <c r="E34" s="136"/>
-      <c r="F34" s="136"/>
-      <c r="G34" s="136"/>
-      <c r="H34" s="136"/>
-      <c r="I34" s="149"/>
-      <c r="J34" s="149"/>
-      <c r="K34" s="136"/>
-      <c r="L34" s="136"/>
-      <c r="M34" s="136"/>
-      <c r="N34" s="136"/>
-      <c r="O34" s="136"/>
-      <c r="P34" s="137"/>
-    </row>
-    <row r="35" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="162" t="s">
+      <c r="B35" s="200"/>
+      <c r="C35" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="163"/>
-      <c r="C35" s="56" t="s">
+      <c r="D35" s="201" t="s">
+        <v>125</v>
+      </c>
+      <c r="E35" s="202"/>
+      <c r="F35" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="D35" s="164"/>
-      <c r="E35" s="165"/>
-      <c r="F35" s="56" t="s">
+      <c r="G35" s="203" t="s">
+        <v>125</v>
+      </c>
+      <c r="H35" s="203"/>
+      <c r="I35" s="204" t="s">
         <v>68</v>
       </c>
-      <c r="G35" s="122"/>
-      <c r="H35" s="122"/>
-      <c r="I35" s="166" t="s">
+      <c r="J35" s="205"/>
+      <c r="K35" s="47" t="s">
+        <v>125</v>
+      </c>
+      <c r="L35" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="J35" s="167"/>
-      <c r="K35" s="47"/>
-      <c r="L35" s="57" t="s">
-        <v>70</v>
-      </c>
-      <c r="M35" s="21"/>
+      <c r="M35" s="21" t="s">
+        <v>125</v>
+      </c>
       <c r="N35" s="25"/>
       <c r="O35" s="57" t="s">
-        <v>71</v>
-      </c>
-      <c r="P35" s="47"/>
+        <v>70</v>
+      </c>
+      <c r="P35" s="47" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="36" spans="1:16" s="49" customFormat="1" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="50"/>
@@ -3292,38 +3351,38 @@
       <c r="P36" s="34"/>
     </row>
     <row r="37" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="148" t="s">
+      <c r="A37" s="216" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="199"/>
+      <c r="C37" s="199"/>
+      <c r="D37" s="199"/>
+      <c r="E37" s="199"/>
+      <c r="F37" s="199"/>
+      <c r="G37" s="199"/>
+      <c r="H37" s="199"/>
+      <c r="I37" s="199"/>
+      <c r="J37" s="199"/>
+      <c r="K37" s="199"/>
+      <c r="L37" s="199"/>
+      <c r="M37" s="199"/>
+      <c r="N37" s="199"/>
+      <c r="O37" s="199"/>
+      <c r="P37" s="217"/>
+    </row>
+    <row r="38" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="218" t="s">
         <v>72</v>
       </c>
-      <c r="B37" s="149"/>
-      <c r="C37" s="149"/>
-      <c r="D37" s="149"/>
-      <c r="E37" s="149"/>
-      <c r="F37" s="149"/>
-      <c r="G37" s="149"/>
-      <c r="H37" s="149"/>
-      <c r="I37" s="149"/>
-      <c r="J37" s="149"/>
-      <c r="K37" s="149"/>
-      <c r="L37" s="149"/>
-      <c r="M37" s="149"/>
-      <c r="N37" s="149"/>
-      <c r="O37" s="149"/>
-      <c r="P37" s="150"/>
-    </row>
-    <row r="38" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="151" t="s">
-        <v>73</v>
-      </c>
-      <c r="B38" s="152"/>
+      <c r="B38" s="219"/>
       <c r="C38" s="58"/>
       <c r="D38" s="59" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E38" s="60"/>
       <c r="F38" s="61"/>
       <c r="G38" s="62" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H38" s="60"/>
       <c r="I38" s="60"/>
@@ -3336,78 +3395,78 @@
       <c r="P38" s="64"/>
     </row>
     <row r="39" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="133"/>
-      <c r="B39" s="153"/>
-      <c r="C39" s="156" t="s">
+      <c r="A39" s="220"/>
+      <c r="B39" s="221"/>
+      <c r="C39" s="165" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39" s="166"/>
+      <c r="E39" s="224"/>
+      <c r="F39" s="224"/>
+      <c r="G39" s="224"/>
+      <c r="H39" s="224"/>
+      <c r="I39" s="224"/>
+      <c r="J39" s="165" t="s">
         <v>76</v>
       </c>
-      <c r="D39" s="157"/>
-      <c r="E39" s="158"/>
-      <c r="F39" s="158"/>
-      <c r="G39" s="158"/>
-      <c r="H39" s="158"/>
-      <c r="I39" s="158"/>
-      <c r="J39" s="156" t="s">
-        <v>77</v>
-      </c>
-      <c r="K39" s="157"/>
+      <c r="K39" s="166"/>
       <c r="L39" s="66"/>
       <c r="M39" s="32" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N39" s="66"/>
-      <c r="O39" s="158"/>
-      <c r="P39" s="159"/>
+      <c r="O39" s="224"/>
+      <c r="P39" s="225"/>
     </row>
     <row r="40" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="154"/>
-      <c r="B40" s="155"/>
+      <c r="A40" s="222"/>
+      <c r="B40" s="223"/>
       <c r="C40" s="126" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" s="127"/>
+      <c r="E40" s="208"/>
+      <c r="F40" s="208"/>
+      <c r="G40" s="208"/>
+      <c r="H40" s="208"/>
+      <c r="I40" s="208"/>
+      <c r="J40" s="126" t="s">
         <v>76</v>
       </c>
-      <c r="D40" s="109"/>
-      <c r="E40" s="146"/>
-      <c r="F40" s="146"/>
-      <c r="G40" s="146"/>
-      <c r="H40" s="146"/>
-      <c r="I40" s="146"/>
-      <c r="J40" s="126" t="s">
-        <v>77</v>
-      </c>
-      <c r="K40" s="109"/>
+      <c r="K40" s="127"/>
       <c r="L40" s="67"/>
       <c r="M40" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="N40" s="67"/>
+      <c r="O40" s="208"/>
+      <c r="P40" s="209"/>
+    </row>
+    <row r="41" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="206" t="s">
         <v>78</v>
       </c>
-      <c r="N40" s="67"/>
-      <c r="O40" s="146"/>
-      <c r="P40" s="147"/>
-    </row>
-    <row r="41" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="144" t="s">
-        <v>79</v>
-      </c>
-      <c r="B41" s="145"/>
-      <c r="C41" s="145"/>
+      <c r="B41" s="207"/>
+      <c r="C41" s="207"/>
       <c r="D41" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="E41" s="146"/>
-      <c r="F41" s="146"/>
-      <c r="G41" s="146"/>
-      <c r="H41" s="146"/>
-      <c r="I41" s="146"/>
-      <c r="J41" s="146"/>
-      <c r="K41" s="146"/>
-      <c r="L41" s="146"/>
-      <c r="M41" s="146"/>
-      <c r="N41" s="146"/>
-      <c r="O41" s="146"/>
-      <c r="P41" s="147"/>
+      <c r="E41" s="208"/>
+      <c r="F41" s="208"/>
+      <c r="G41" s="208"/>
+      <c r="H41" s="208"/>
+      <c r="I41" s="208"/>
+      <c r="J41" s="208"/>
+      <c r="K41" s="208"/>
+      <c r="L41" s="208"/>
+      <c r="M41" s="208"/>
+      <c r="N41" s="208"/>
+      <c r="O41" s="208"/>
+      <c r="P41" s="209"/>
     </row>
     <row r="42" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="69" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D42" s="70"/>
       <c r="E42" s="71"/>
@@ -3445,162 +3504,162 @@
       <c r="P44" s="71"/>
     </row>
     <row r="45" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="135" t="s">
+      <c r="A45" s="111" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45" s="112"/>
+      <c r="C45" s="112"/>
+      <c r="D45" s="112"/>
+      <c r="E45" s="112"/>
+      <c r="F45" s="112"/>
+      <c r="G45" s="112"/>
+      <c r="H45" s="112"/>
+      <c r="I45" s="112"/>
+      <c r="J45" s="112"/>
+      <c r="K45" s="112"/>
+      <c r="L45" s="112"/>
+      <c r="M45" s="112"/>
+      <c r="N45" s="112"/>
+      <c r="O45" s="112"/>
+      <c r="P45" s="113"/>
+    </row>
+    <row r="46" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="210" t="s">
         <v>81</v>
       </c>
-      <c r="B45" s="136"/>
-      <c r="C45" s="136"/>
-      <c r="D45" s="136"/>
-      <c r="E45" s="136"/>
-      <c r="F45" s="136"/>
-      <c r="G45" s="136"/>
-      <c r="H45" s="136"/>
-      <c r="I45" s="136"/>
-      <c r="J45" s="136"/>
-      <c r="K45" s="136"/>
-      <c r="L45" s="136"/>
-      <c r="M45" s="136"/>
-      <c r="N45" s="136"/>
-      <c r="O45" s="136"/>
-      <c r="P45" s="137"/>
-    </row>
-    <row r="46" spans="1:16" s="65" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="113" t="s">
+      <c r="B46" s="211"/>
+      <c r="C46" s="211"/>
+      <c r="D46" s="211"/>
+      <c r="E46" s="211"/>
+      <c r="F46" s="211"/>
+      <c r="G46" s="211"/>
+      <c r="H46" s="210" t="s">
         <v>82</v>
       </c>
-      <c r="B46" s="114"/>
-      <c r="C46" s="114"/>
-      <c r="D46" s="114"/>
-      <c r="E46" s="114"/>
-      <c r="F46" s="114"/>
-      <c r="G46" s="114"/>
-      <c r="H46" s="113" t="s">
+      <c r="I46" s="211"/>
+      <c r="J46" s="211"/>
+      <c r="K46" s="211"/>
+      <c r="L46" s="211"/>
+      <c r="M46" s="211"/>
+      <c r="N46" s="211"/>
+      <c r="O46" s="211"/>
+      <c r="P46" s="212"/>
+    </row>
+    <row r="47" spans="1:16" s="65" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="213" t="s">
         <v>83</v>
-      </c>
-      <c r="I46" s="114"/>
-      <c r="J46" s="114"/>
-      <c r="K46" s="114"/>
-      <c r="L46" s="114"/>
-      <c r="M46" s="114"/>
-      <c r="N46" s="114"/>
-      <c r="O46" s="114"/>
-      <c r="P46" s="115"/>
-    </row>
-    <row r="47" spans="1:16" s="65" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="130" t="s">
-        <v>84</v>
       </c>
       <c r="B47" s="78"/>
       <c r="C47" s="79" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D47" s="78"/>
       <c r="E47" s="79" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F47" s="78"/>
       <c r="G47" s="80" t="s">
+        <v>86</v>
+      </c>
+      <c r="H47" s="81" t="s">
         <v>87</v>
-      </c>
-      <c r="H47" s="81" t="s">
-        <v>88</v>
       </c>
       <c r="I47" s="78"/>
       <c r="J47" s="79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K47" s="78"/>
       <c r="L47" s="79" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M47" s="78"/>
       <c r="N47" s="79" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O47" s="82"/>
       <c r="P47" s="83" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:16" s="65" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="131"/>
+      <c r="A48" s="214"/>
       <c r="B48" s="78"/>
       <c r="C48" s="84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D48" s="78"/>
       <c r="E48" s="84" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F48" s="78"/>
       <c r="G48" s="85" t="s">
+        <v>94</v>
+      </c>
+      <c r="H48" s="86" t="s">
         <v>95</v>
-      </c>
-      <c r="H48" s="86" t="s">
-        <v>96</v>
       </c>
       <c r="I48" s="78"/>
       <c r="J48" s="84" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K48" s="78"/>
       <c r="L48" s="84" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M48" s="78"/>
       <c r="N48" s="84" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O48" s="82"/>
       <c r="P48" s="87" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="1:16" s="65" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="132"/>
+      <c r="A49" s="215"/>
       <c r="B49" s="78"/>
       <c r="C49" s="88" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D49" s="78"/>
       <c r="E49" s="89" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F49" s="89"/>
       <c r="G49" s="90"/>
       <c r="H49" s="86" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I49" s="78"/>
       <c r="J49" s="84" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K49" s="78"/>
       <c r="L49" s="84" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M49" s="78"/>
       <c r="N49" s="84" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O49" s="71"/>
       <c r="P49" s="87"/>
     </row>
     <row r="50" spans="1:16" s="65" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="130" t="s">
-        <v>100</v>
+      <c r="A50" s="213" t="s">
+        <v>99</v>
       </c>
       <c r="B50" s="78"/>
       <c r="C50" s="84" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D50" s="91"/>
       <c r="E50" s="84" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F50" s="91"/>
       <c r="G50" s="85" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H50" s="92"/>
       <c r="I50" s="84"/>
@@ -3613,23 +3672,23 @@
       <c r="P50" s="87"/>
     </row>
     <row r="51" spans="1:16" s="65" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="131"/>
+      <c r="A51" s="214"/>
       <c r="B51" s="78"/>
       <c r="C51" s="84" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D51" s="78"/>
       <c r="E51" s="84" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F51" s="78"/>
       <c r="G51" s="85" t="s">
+        <v>105</v>
+      </c>
+      <c r="H51" s="220" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="133" t="s">
-        <v>107</v>
-      </c>
-      <c r="I51" s="134"/>
+      <c r="I51" s="239"/>
       <c r="J51" s="78"/>
       <c r="K51" s="84"/>
       <c r="L51" s="84"/>
@@ -3639,14 +3698,14 @@
       <c r="P51" s="87"/>
     </row>
     <row r="52" spans="1:16" s="65" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="132"/>
+      <c r="A52" s="215"/>
       <c r="B52" s="93"/>
       <c r="C52" s="74" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D52" s="94"/>
       <c r="E52" s="75" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F52" s="74"/>
       <c r="G52" s="95"/>
@@ -3674,124 +3733,124 @@
       <c r="P53" s="71"/>
     </row>
     <row r="54" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="135" t="s">
+      <c r="A54" s="111" t="s">
+        <v>109</v>
+      </c>
+      <c r="B54" s="112"/>
+      <c r="C54" s="112"/>
+      <c r="D54" s="112"/>
+      <c r="E54" s="112"/>
+      <c r="F54" s="112"/>
+      <c r="G54" s="112"/>
+      <c r="H54" s="112"/>
+      <c r="I54" s="112"/>
+      <c r="J54" s="112"/>
+      <c r="K54" s="112"/>
+      <c r="L54" s="112"/>
+      <c r="M54" s="112"/>
+      <c r="N54" s="112"/>
+      <c r="O54" s="112"/>
+      <c r="P54" s="113"/>
+    </row>
+    <row r="55" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="137" t="s">
         <v>110</v>
       </c>
-      <c r="B54" s="136"/>
-      <c r="C54" s="136"/>
-      <c r="D54" s="136"/>
-      <c r="E54" s="136"/>
-      <c r="F54" s="136"/>
-      <c r="G54" s="136"/>
-      <c r="H54" s="136"/>
-      <c r="I54" s="136"/>
-      <c r="J54" s="136"/>
-      <c r="K54" s="136"/>
-      <c r="L54" s="136"/>
-      <c r="M54" s="136"/>
-      <c r="N54" s="136"/>
-      <c r="O54" s="136"/>
-      <c r="P54" s="137"/>
-    </row>
-    <row r="55" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="138" t="s">
+      <c r="B55" s="181"/>
+      <c r="C55" s="181"/>
+      <c r="D55" s="191"/>
+      <c r="E55" s="179"/>
+      <c r="F55" s="126" t="s">
         <v>111</v>
       </c>
-      <c r="B55" s="139"/>
-      <c r="C55" s="139"/>
-      <c r="D55" s="140"/>
-      <c r="E55" s="141"/>
-      <c r="F55" s="126" t="s">
+      <c r="G55" s="127"/>
+      <c r="H55" s="141"/>
+      <c r="I55" s="141"/>
+      <c r="J55" s="141"/>
+      <c r="K55" s="141"/>
+      <c r="L55" s="141"/>
+      <c r="M55" s="141"/>
+      <c r="N55" s="141"/>
+      <c r="O55" s="141"/>
+      <c r="P55" s="240"/>
+    </row>
+    <row r="56" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="121" t="s">
         <v>112</v>
       </c>
-      <c r="G55" s="109"/>
-      <c r="H55" s="142"/>
-      <c r="I55" s="142"/>
-      <c r="J55" s="142"/>
-      <c r="K55" s="142"/>
-      <c r="L55" s="142"/>
-      <c r="M55" s="142"/>
-      <c r="N55" s="142"/>
-      <c r="O55" s="142"/>
-      <c r="P55" s="143"/>
-    </row>
-    <row r="56" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="108" t="s">
+      <c r="B56" s="127"/>
+      <c r="C56" s="127"/>
+      <c r="D56" s="182"/>
+      <c r="E56" s="183"/>
+      <c r="F56" s="126" t="s">
         <v>113</v>
       </c>
-      <c r="B56" s="109"/>
-      <c r="C56" s="109"/>
-      <c r="D56" s="124"/>
-      <c r="E56" s="125"/>
-      <c r="F56" s="126" t="s">
-        <v>114</v>
-      </c>
-      <c r="G56" s="109"/>
-      <c r="H56" s="109"/>
+      <c r="G56" s="127"/>
+      <c r="H56" s="127"/>
       <c r="I56" s="97"/>
-      <c r="J56" s="124"/>
-      <c r="K56" s="124"/>
+      <c r="J56" s="182"/>
+      <c r="K56" s="182"/>
       <c r="L56" s="97"/>
-      <c r="M56" s="124"/>
-      <c r="N56" s="124"/>
+      <c r="M56" s="182"/>
+      <c r="N56" s="182"/>
       <c r="O56" s="11"/>
       <c r="P56" s="13"/>
     </row>
     <row r="57" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="108" t="s">
+      <c r="A57" s="121" t="s">
+        <v>114</v>
+      </c>
+      <c r="B57" s="127"/>
+      <c r="C57" s="236"/>
+      <c r="D57" s="237"/>
+      <c r="E57" s="238"/>
+      <c r="F57" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="B57" s="109"/>
-      <c r="C57" s="127"/>
-      <c r="D57" s="128"/>
-      <c r="E57" s="129"/>
-      <c r="F57" s="35" t="s">
+      <c r="G57" s="227"/>
+      <c r="H57" s="227"/>
+      <c r="I57" s="227"/>
+      <c r="J57" s="227"/>
+      <c r="K57" s="227"/>
+      <c r="L57" s="227"/>
+      <c r="M57" s="227"/>
+      <c r="N57" s="227"/>
+      <c r="O57" s="227"/>
+      <c r="P57" s="228"/>
+    </row>
+    <row r="58" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="121" t="s">
         <v>116</v>
       </c>
-      <c r="G57" s="111"/>
-      <c r="H57" s="111"/>
-      <c r="I57" s="111"/>
-      <c r="J57" s="111"/>
-      <c r="K57" s="111"/>
-      <c r="L57" s="111"/>
-      <c r="M57" s="111"/>
-      <c r="N57" s="111"/>
-      <c r="O57" s="111"/>
-      <c r="P57" s="112"/>
-    </row>
-    <row r="58" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="108" t="s">
-        <v>117</v>
-      </c>
-      <c r="B58" s="109"/>
-      <c r="C58" s="110"/>
-      <c r="D58" s="111"/>
-      <c r="E58" s="111"/>
-      <c r="F58" s="111"/>
-      <c r="G58" s="111"/>
-      <c r="H58" s="111"/>
-      <c r="I58" s="111"/>
-      <c r="J58" s="111"/>
-      <c r="K58" s="111"/>
-      <c r="L58" s="111"/>
-      <c r="M58" s="111"/>
-      <c r="N58" s="111"/>
-      <c r="O58" s="111"/>
-      <c r="P58" s="112"/>
+      <c r="B58" s="127"/>
+      <c r="C58" s="226"/>
+      <c r="D58" s="227"/>
+      <c r="E58" s="227"/>
+      <c r="F58" s="227"/>
+      <c r="G58" s="227"/>
+      <c r="H58" s="227"/>
+      <c r="I58" s="227"/>
+      <c r="J58" s="227"/>
+      <c r="K58" s="227"/>
+      <c r="L58" s="227"/>
+      <c r="M58" s="227"/>
+      <c r="N58" s="227"/>
+      <c r="O58" s="227"/>
+      <c r="P58" s="228"/>
     </row>
     <row r="59" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="98" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B59" s="99"/>
       <c r="C59" s="25"/>
       <c r="D59" s="100" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E59" s="100"/>
       <c r="F59" s="25"/>
       <c r="G59" s="100" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H59" s="100"/>
       <c r="I59" s="100"/>
@@ -3805,35 +3864,35 @@
     </row>
     <row r="60" spans="1:16" s="49" customFormat="1" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="61" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="113" t="s">
-        <v>119</v>
-      </c>
-      <c r="B61" s="114"/>
-      <c r="C61" s="114"/>
-      <c r="D61" s="114"/>
-      <c r="E61" s="114"/>
-      <c r="F61" s="114"/>
-      <c r="G61" s="114"/>
-      <c r="H61" s="114"/>
-      <c r="I61" s="114"/>
-      <c r="J61" s="114"/>
-      <c r="K61" s="114"/>
-      <c r="L61" s="114"/>
-      <c r="M61" s="114"/>
-      <c r="N61" s="114"/>
-      <c r="O61" s="114"/>
-      <c r="P61" s="115"/>
+      <c r="A61" s="210" t="s">
+        <v>118</v>
+      </c>
+      <c r="B61" s="211"/>
+      <c r="C61" s="211"/>
+      <c r="D61" s="211"/>
+      <c r="E61" s="211"/>
+      <c r="F61" s="211"/>
+      <c r="G61" s="211"/>
+      <c r="H61" s="211"/>
+      <c r="I61" s="211"/>
+      <c r="J61" s="211"/>
+      <c r="K61" s="211"/>
+      <c r="L61" s="211"/>
+      <c r="M61" s="211"/>
+      <c r="N61" s="211"/>
+      <c r="O61" s="211"/>
+      <c r="P61" s="212"/>
     </row>
     <row r="62" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A62" s="93"/>
       <c r="B62" s="102" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C62" s="102"/>
       <c r="D62" s="102"/>
       <c r="E62" s="93"/>
       <c r="F62" s="102" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G62" s="102"/>
       <c r="H62" s="93"/>
@@ -3849,7 +3908,7 @@
     <row r="63" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="93"/>
       <c r="B63" s="104" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C63" s="104"/>
       <c r="D63" s="104"/>
@@ -3869,7 +3928,7 @@
     <row r="64" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="93"/>
       <c r="B64" s="102" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C64" s="102"/>
       <c r="D64" s="102"/>
@@ -3889,7 +3948,7 @@
     <row r="65" spans="1:16" s="49" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="93"/>
       <c r="B65" s="106" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C65" s="106"/>
       <c r="D65" s="106"/>
@@ -3907,43 +3966,153 @@
       <c r="P65" s="107"/>
     </row>
     <row r="66" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="116"/>
-      <c r="B66" s="117"/>
-      <c r="C66" s="117"/>
-      <c r="D66" s="117"/>
-      <c r="E66" s="116"/>
-      <c r="F66" s="117"/>
-      <c r="G66" s="117"/>
-      <c r="H66" s="116"/>
-      <c r="I66" s="117"/>
-      <c r="J66" s="117"/>
-      <c r="K66" s="116"/>
-      <c r="L66" s="117"/>
-      <c r="M66" s="117"/>
-      <c r="N66" s="117"/>
-      <c r="O66" s="117"/>
-      <c r="P66" s="117"/>
+      <c r="A66" s="229"/>
+      <c r="B66" s="230"/>
+      <c r="C66" s="230"/>
+      <c r="D66" s="230"/>
+      <c r="E66" s="229"/>
+      <c r="F66" s="230"/>
+      <c r="G66" s="230"/>
+      <c r="H66" s="229"/>
+      <c r="I66" s="230"/>
+      <c r="J66" s="230"/>
+      <c r="K66" s="229"/>
+      <c r="L66" s="230"/>
+      <c r="M66" s="230"/>
+      <c r="N66" s="230"/>
+      <c r="O66" s="230"/>
+      <c r="P66" s="230"/>
     </row>
     <row r="67" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="117"/>
-      <c r="B67" s="117"/>
-      <c r="C67" s="117"/>
-      <c r="D67" s="117"/>
-      <c r="E67" s="117"/>
-      <c r="F67" s="117"/>
-      <c r="G67" s="117"/>
-      <c r="H67" s="117"/>
-      <c r="I67" s="117"/>
-      <c r="J67" s="117"/>
-      <c r="K67" s="117"/>
-      <c r="L67" s="117"/>
-      <c r="M67" s="117"/>
-      <c r="N67" s="117"/>
-      <c r="O67" s="117"/>
-      <c r="P67" s="117"/>
+      <c r="A67" s="230"/>
+      <c r="B67" s="230"/>
+      <c r="C67" s="230"/>
+      <c r="D67" s="230"/>
+      <c r="E67" s="230"/>
+      <c r="F67" s="230"/>
+      <c r="G67" s="230"/>
+      <c r="H67" s="230"/>
+      <c r="I67" s="230"/>
+      <c r="J67" s="230"/>
+      <c r="K67" s="230"/>
+      <c r="L67" s="230"/>
+      <c r="M67" s="230"/>
+      <c r="N67" s="230"/>
+      <c r="O67" s="230"/>
+      <c r="P67" s="230"/>
     </row>
   </sheetData>
   <mergeCells count="134">
+    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="D58:P58"/>
+    <mergeCell ref="A61:P61"/>
+    <mergeCell ref="A66:P66"/>
+    <mergeCell ref="A67:P67"/>
+    <mergeCell ref="C5:P5"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="F56:H56"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="M56:N56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="G57:P57"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="H55:P55"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="E41:P41"/>
+    <mergeCell ref="A45:P45"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="H46:P46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A37:P37"/>
+    <mergeCell ref="A38:B40"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:I39"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:I40"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="H32:P32"/>
+    <mergeCell ref="A34:P34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="K28:M28"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:P29"/>
+    <mergeCell ref="A26:P26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="A21:B24"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="A19:B20"/>
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:P13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:P14"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="A5:B5"/>
@@ -3968,116 +4137,6 @@
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="A16:B17"/>
     <mergeCell ref="D16:F16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="C13:P13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:P14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="A19:B20"/>
-    <mergeCell ref="D19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="A21:B24"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="K28:M28"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:P29"/>
-    <mergeCell ref="A26:P26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="H32:P32"/>
-    <mergeCell ref="A34:P34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="E41:P41"/>
-    <mergeCell ref="A45:P45"/>
-    <mergeCell ref="A46:G46"/>
-    <mergeCell ref="H46:P46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A37:P37"/>
-    <mergeCell ref="A38:B40"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:I39"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:I40"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="O40:P40"/>
-    <mergeCell ref="A58:C58"/>
-    <mergeCell ref="D58:P58"/>
-    <mergeCell ref="A61:P61"/>
-    <mergeCell ref="A66:P66"/>
-    <mergeCell ref="A67:P67"/>
-    <mergeCell ref="C5:P5"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="A56:C56"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="F56:H56"/>
-    <mergeCell ref="J56:K56"/>
-    <mergeCell ref="M56:N56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="G57:P57"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="H51:I51"/>
-    <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="H55:P55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>